<commit_message>
v9.53: package Waves 1–5 build + refresh registry audit
Repackaged runnable build QueryBook-v9.53-2026-10-02.zip with all five waves
(no secrets/local state). Refreshed the registry audit to reflect the new
backends: Included rose 29 → 68, Missing fell 150 → 120 (30 features promoted
across LIL, PIL, query understanding, response ranking, ontology, assessment,
rights, UIAS, provenance lineage, webhooks).

docs/QueryBook-Prototype-Registry-Audit.xlsx and
docs/QueryBook-Prototype-Registry-Checklist.docx regenerated (v9.53 label).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019szkZU7hLaBcGBEqVSVWY6
</commit_message>
<xml_diff>
--- a/docs/QueryBook-Prototype-Registry-Audit.xlsx
+++ b/docs/QueryBook-Prototype-Registry-Audit.xlsx
@@ -576,7 +576,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Prototype: QueryBook v9.51  ·  Registry: 219 enumerated features  ·  Date: 2026-10-02</t>
+          <t>Prototype: QueryBook v9.53  ·  Registry: 219 enumerated features  ·  Date: 2026-10-02</t>
         </is>
       </c>
     </row>
@@ -611,10 +611,10 @@
         </is>
       </c>
       <c r="B6" s="6" t="n">
-        <v>29</v>
+        <v>68</v>
       </c>
       <c r="C6" s="6" t="n">
-        <v>13.2</v>
+        <v>31.1</v>
       </c>
     </row>
     <row r="7">
@@ -624,10 +624,10 @@
         </is>
       </c>
       <c r="B7" s="8" t="n">
-        <v>40</v>
+        <v>31</v>
       </c>
       <c r="C7" s="8" t="n">
-        <v>18.3</v>
+        <v>14.2</v>
       </c>
     </row>
     <row r="8">
@@ -637,10 +637,10 @@
         </is>
       </c>
       <c r="B8" s="10" t="n">
-        <v>150</v>
+        <v>120</v>
       </c>
       <c r="C8" s="10" t="n">
-        <v>68.5</v>
+        <v>54.8</v>
       </c>
     </row>
     <row r="9">
@@ -659,7 +659,7 @@
     <row r="11">
       <c r="A11" s="12" t="inlineStr">
         <is>
-          <t>Reading: the prototype fully supports 29 features and partially supports 40 (= 69 of 219, 32% touched); 150 are not present.</t>
+          <t>Reading: the prototype fully supports 68 features and partially supports 31 (= 99 of 219, 45% touched); 120 are not present.</t>
         </is>
       </c>
     </row>
@@ -761,10 +761,10 @@
         </is>
       </c>
       <c r="B18" s="13" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="C18" s="13" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="D18" s="13" t="n">
         <v>1</v>
@@ -780,13 +780,13 @@
         </is>
       </c>
       <c r="B19" s="13" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="C19" s="13" t="n">
         <v>0</v>
       </c>
       <c r="D19" s="13" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="E19" s="13" t="n">
         <v>13</v>
@@ -799,13 +799,13 @@
         </is>
       </c>
       <c r="B20" s="13" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="C20" s="13" t="n">
         <v>0</v>
       </c>
       <c r="D20" s="13" t="n">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="E20" s="13" t="n">
         <v>16</v>
@@ -818,13 +818,13 @@
         </is>
       </c>
       <c r="B21" s="13" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="C21" s="13" t="n">
         <v>0</v>
       </c>
       <c r="D21" s="13" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="E21" s="13" t="n">
         <v>12</v>
@@ -837,13 +837,13 @@
         </is>
       </c>
       <c r="B22" s="13" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C22" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D22" s="13" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="E22" s="13" t="n">
         <v>10</v>
@@ -856,13 +856,13 @@
         </is>
       </c>
       <c r="B23" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C23" s="13" t="n">
         <v>1</v>
       </c>
       <c r="D23" s="13" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E23" s="13" t="n">
         <v>12</v>
@@ -913,10 +913,10 @@
         </is>
       </c>
       <c r="B26" s="13" t="n">
+        <v>6</v>
+      </c>
+      <c r="C26" s="13" t="n">
         <v>3</v>
-      </c>
-      <c r="C26" s="13" t="n">
-        <v>6</v>
       </c>
       <c r="D26" s="13" t="n">
         <v>1</v>
@@ -951,13 +951,13 @@
         </is>
       </c>
       <c r="B28" s="13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C28" s="13" t="n">
         <v>4</v>
       </c>
       <c r="D28" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E28" s="13" t="n">
         <v>5</v>
@@ -1008,13 +1008,13 @@
         </is>
       </c>
       <c r="B31" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="C31" s="13" t="n">
+        <v>2</v>
+      </c>
+      <c r="D31" s="13" t="n">
         <v>0</v>
-      </c>
-      <c r="C31" s="13" t="n">
-        <v>3</v>
-      </c>
-      <c r="D31" s="13" t="n">
-        <v>2</v>
       </c>
       <c r="E31" s="13" t="n">
         <v>5</v>
@@ -1027,13 +1027,13 @@
         </is>
       </c>
       <c r="B32" s="13" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="C32" s="13" t="n">
         <v>0</v>
       </c>
       <c r="D32" s="13" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="E32" s="13" t="n">
         <v>6</v>
@@ -1046,13 +1046,13 @@
         </is>
       </c>
       <c r="B33" s="13" t="n">
+        <v>4</v>
+      </c>
+      <c r="C33" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="D33" s="13" t="n">
         <v>1</v>
-      </c>
-      <c r="C33" s="13" t="n">
-        <v>1</v>
-      </c>
-      <c r="D33" s="13" t="n">
-        <v>3</v>
       </c>
       <c r="E33" s="13" t="n">
         <v>5</v>
@@ -1084,13 +1084,13 @@
         </is>
       </c>
       <c r="B35" s="11" t="n">
-        <v>29</v>
+        <v>68</v>
       </c>
       <c r="C35" s="11" t="n">
-        <v>40</v>
+        <v>31</v>
       </c>
       <c r="D35" s="11" t="n">
-        <v>150</v>
+        <v>120</v>
       </c>
       <c r="E35" s="11" t="n">
         <v>219</v>
@@ -3425,24 +3425,24 @@
           <t>4. Query Understanding</t>
         </is>
       </c>
-      <c r="D60" s="19" t="inlineStr">
-        <is>
-          <t>Partial</t>
-        </is>
-      </c>
-      <c r="E60" s="20" t="inlineStr">
-        <is>
-          <t>~</t>
+      <c r="D60" s="23" t="inlineStr">
+        <is>
+          <t>Included</t>
+        </is>
+      </c>
+      <c r="E60" s="24" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="F60" s="17" t="inlineStr">
         <is>
-          <t>qb_chat.retrieve/plan_queries</t>
+          <t>qb_query.entities</t>
         </is>
       </c>
       <c r="G60" s="17" t="inlineStr">
         <is>
-          <t>Entities are matched during retrieval; no standalone resolver.</t>
+          <t>Deterministic entity extraction.</t>
         </is>
       </c>
       <c r="H60" s="17" t="inlineStr"/>
@@ -3461,24 +3461,24 @@
           <t>4. Query Understanding</t>
         </is>
       </c>
-      <c r="D61" s="19" t="inlineStr">
-        <is>
-          <t>Partial</t>
-        </is>
-      </c>
-      <c r="E61" s="20" t="inlineStr">
-        <is>
-          <t>~</t>
+      <c r="D61" s="23" t="inlineStr">
+        <is>
+          <t>Included</t>
+        </is>
+      </c>
+      <c r="E61" s="24" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="F61" s="17" t="inlineStr">
         <is>
-          <t>ufcs_store.fql (predicate match)</t>
+          <t>qb_query.predicate</t>
         </is>
       </c>
       <c r="G61" s="17" t="inlineStr">
         <is>
-          <t>Predicates are modeled and matched in FQL.</t>
+          <t>Predicate resolution via cue table + FQL.</t>
         </is>
       </c>
       <c r="H61" s="17" t="inlineStr"/>
@@ -3497,24 +3497,24 @@
           <t>4. Query Understanding</t>
         </is>
       </c>
-      <c r="D62" s="19" t="inlineStr">
-        <is>
-          <t>Partial</t>
-        </is>
-      </c>
-      <c r="E62" s="20" t="inlineStr">
-        <is>
-          <t>~</t>
+      <c r="D62" s="23" t="inlineStr">
+        <is>
+          <t>Included</t>
+        </is>
+      </c>
+      <c r="E62" s="24" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="F62" s="17" t="inlineStr">
         <is>
-          <t>qb_chat.plan_queries/gate</t>
+          <t>qb_query.intent</t>
         </is>
       </c>
       <c r="G62" s="17" t="inlineStr">
         <is>
-          <t>Query intent is planned in the chat pipeline.</t>
+          <t>Intent classification (question/command/statement).</t>
         </is>
       </c>
       <c r="H62" s="17" t="inlineStr"/>
@@ -3569,24 +3569,24 @@
           <t>4. Query Understanding</t>
         </is>
       </c>
-      <c r="D64" s="19" t="inlineStr">
-        <is>
-          <t>Partial</t>
-        </is>
-      </c>
-      <c r="E64" s="20" t="inlineStr">
-        <is>
-          <t>~</t>
+      <c r="D64" s="23" t="inlineStr">
+        <is>
+          <t>Included</t>
+        </is>
+      </c>
+      <c r="E64" s="24" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="F64" s="17" t="inlineStr">
         <is>
-          <t>/api/domains, /api/domain_logic</t>
+          <t>qb_query.understand (scope)</t>
         </is>
       </c>
       <c r="G64" s="17" t="inlineStr">
         <is>
-          <t>Domain scoping exists; not a full scope-detection engine.</t>
+          <t>Scope set in the query plan.</t>
         </is>
       </c>
       <c r="H64" s="17" t="inlineStr"/>
@@ -3637,24 +3637,24 @@
           <t>4. Query Understanding</t>
         </is>
       </c>
-      <c r="D66" s="19" t="inlineStr">
-        <is>
-          <t>Partial</t>
-        </is>
-      </c>
-      <c r="E66" s="20" t="inlineStr">
-        <is>
-          <t>~</t>
+      <c r="D66" s="23" t="inlineStr">
+        <is>
+          <t>Included</t>
+        </is>
+      </c>
+      <c r="E66" s="24" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="F66" s="17" t="inlineStr">
         <is>
-          <t>qb_chat.plan_queries</t>
+          <t>qb_query.expand</t>
         </is>
       </c>
       <c r="G66" s="17" t="inlineStr">
         <is>
-          <t>The planner expands a question into multiple store queries.</t>
+          <t>Deterministic query expansion.</t>
         </is>
       </c>
       <c r="H66" s="17" t="inlineStr"/>
@@ -3745,20 +3745,24 @@
           <t>5. Ontology / Concept Graph</t>
         </is>
       </c>
-      <c r="D69" s="21" t="inlineStr">
-        <is>
-          <t>Missing</t>
-        </is>
-      </c>
-      <c r="E69" s="22" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="F69" s="17" t="inlineStr"/>
+      <c r="D69" s="23" t="inlineStr">
+        <is>
+          <t>Included</t>
+        </is>
+      </c>
+      <c r="E69" s="24" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F69" s="17" t="inlineStr">
+        <is>
+          <t>qb_ontology.build</t>
+        </is>
+      </c>
       <c r="G69" s="17" t="inlineStr">
         <is>
-          <t>No ontology DAG / concept-node / edge subsystem in the prototype.</t>
+          <t>Concept graph (DAG-style) from Fact-Unit triples.</t>
         </is>
       </c>
       <c r="H69" s="17" t="inlineStr"/>
@@ -3777,20 +3781,24 @@
           <t>5. Ontology / Concept Graph</t>
         </is>
       </c>
-      <c r="D70" s="21" t="inlineStr">
-        <is>
-          <t>Missing</t>
-        </is>
-      </c>
-      <c r="E70" s="22" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="F70" s="17" t="inlineStr"/>
+      <c r="D70" s="23" t="inlineStr">
+        <is>
+          <t>Included</t>
+        </is>
+      </c>
+      <c r="E70" s="24" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F70" s="17" t="inlineStr">
+        <is>
+          <t>qb_ontology (nodes)</t>
+        </is>
+      </c>
       <c r="G70" s="17" t="inlineStr">
         <is>
-          <t>No ontology DAG / concept-node / edge subsystem in the prototype.</t>
+          <t>Concept nodes.</t>
         </is>
       </c>
       <c r="H70" s="17" t="inlineStr"/>
@@ -3809,20 +3817,24 @@
           <t>5. Ontology / Concept Graph</t>
         </is>
       </c>
-      <c r="D71" s="21" t="inlineStr">
-        <is>
-          <t>Missing</t>
-        </is>
-      </c>
-      <c r="E71" s="22" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="F71" s="17" t="inlineStr"/>
+      <c r="D71" s="23" t="inlineStr">
+        <is>
+          <t>Included</t>
+        </is>
+      </c>
+      <c r="E71" s="24" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F71" s="17" t="inlineStr">
+        <is>
+          <t>qb_ontology (hierarchical edges)</t>
+        </is>
+      </c>
       <c r="G71" s="17" t="inlineStr">
         <is>
-          <t>No ontology DAG / concept-node / edge subsystem in the prototype.</t>
+          <t>Hierarchical edges.</t>
         </is>
       </c>
       <c r="H71" s="17" t="inlineStr"/>
@@ -3841,20 +3853,24 @@
           <t>5. Ontology / Concept Graph</t>
         </is>
       </c>
-      <c r="D72" s="21" t="inlineStr">
-        <is>
-          <t>Missing</t>
-        </is>
-      </c>
-      <c r="E72" s="22" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="F72" s="17" t="inlineStr"/>
+      <c r="D72" s="23" t="inlineStr">
+        <is>
+          <t>Included</t>
+        </is>
+      </c>
+      <c r="E72" s="24" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F72" s="17" t="inlineStr">
+        <is>
+          <t>qb_ontology (prerequisite edges)</t>
+        </is>
+      </c>
       <c r="G72" s="17" t="inlineStr">
         <is>
-          <t>No ontology DAG / concept-node / edge subsystem in the prototype.</t>
+          <t>Prerequisite edges.</t>
         </is>
       </c>
       <c r="H72" s="17" t="inlineStr"/>
@@ -3873,20 +3889,24 @@
           <t>5. Ontology / Concept Graph</t>
         </is>
       </c>
-      <c r="D73" s="21" t="inlineStr">
-        <is>
-          <t>Missing</t>
-        </is>
-      </c>
-      <c r="E73" s="22" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="F73" s="17" t="inlineStr"/>
+      <c r="D73" s="23" t="inlineStr">
+        <is>
+          <t>Included</t>
+        </is>
+      </c>
+      <c r="E73" s="24" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F73" s="17" t="inlineStr">
+        <is>
+          <t>qb_ontology (equivalence edges)</t>
+        </is>
+      </c>
       <c r="G73" s="17" t="inlineStr">
         <is>
-          <t>No ontology DAG / concept-node / edge subsystem in the prototype.</t>
+          <t>Equivalence edges.</t>
         </is>
       </c>
       <c r="H73" s="17" t="inlineStr"/>
@@ -3905,20 +3925,24 @@
           <t>5. Ontology / Concept Graph</t>
         </is>
       </c>
-      <c r="D74" s="21" t="inlineStr">
-        <is>
-          <t>Missing</t>
-        </is>
-      </c>
-      <c r="E74" s="22" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="F74" s="17" t="inlineStr"/>
+      <c r="D74" s="23" t="inlineStr">
+        <is>
+          <t>Included</t>
+        </is>
+      </c>
+      <c r="E74" s="24" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F74" s="17" t="inlineStr">
+        <is>
+          <t>qb_ontology.concept_path</t>
+        </is>
+      </c>
       <c r="G74" s="17" t="inlineStr">
         <is>
-          <t>No ontology DAG / concept-node / edge subsystem in the prototype.</t>
+          <t>Concept path generator (BFS).</t>
         </is>
       </c>
       <c r="H74" s="17" t="inlineStr"/>
@@ -4161,20 +4185,24 @@
           <t>6. Assessment / Education</t>
         </is>
       </c>
-      <c r="D82" s="21" t="inlineStr">
-        <is>
-          <t>Missing</t>
-        </is>
-      </c>
-      <c r="E82" s="22" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="F82" s="17" t="inlineStr"/>
+      <c r="D82" s="23" t="inlineStr">
+        <is>
+          <t>Included</t>
+        </is>
+      </c>
+      <c r="E82" s="24" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F82" s="17" t="inlineStr">
+        <is>
+          <t>qb_assess.items_from_triples</t>
+        </is>
+      </c>
       <c r="G82" s="17" t="inlineStr">
         <is>
-          <t>No assessment/education subsystem in the prototype.</t>
+          <t>Assessment item generator.</t>
         </is>
       </c>
       <c r="H82" s="17" t="inlineStr"/>
@@ -4193,20 +4221,24 @@
           <t>6. Assessment / Education</t>
         </is>
       </c>
-      <c r="D83" s="21" t="inlineStr">
-        <is>
-          <t>Missing</t>
-        </is>
-      </c>
-      <c r="E83" s="22" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="F83" s="17" t="inlineStr"/>
+      <c r="D83" s="23" t="inlineStr">
+        <is>
+          <t>Included</t>
+        </is>
+      </c>
+      <c r="E83" s="24" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F83" s="17" t="inlineStr">
+        <is>
+          <t>qb_assess (distractors)</t>
+        </is>
+      </c>
       <c r="G83" s="17" t="inlineStr">
         <is>
-          <t>No assessment/education subsystem in the prototype.</t>
+          <t>Same-predicate distractor generator.</t>
         </is>
       </c>
       <c r="H83" s="17" t="inlineStr"/>
@@ -4225,20 +4257,24 @@
           <t>6. Assessment / Education</t>
         </is>
       </c>
-      <c r="D84" s="21" t="inlineStr">
-        <is>
-          <t>Missing</t>
-        </is>
-      </c>
-      <c r="E84" s="22" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="F84" s="17" t="inlineStr"/>
+      <c r="D84" s="23" t="inlineStr">
+        <is>
+          <t>Included</t>
+        </is>
+      </c>
+      <c r="E84" s="24" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F84" s="17" t="inlineStr">
+        <is>
+          <t>qb_assess (competency)</t>
+        </is>
+      </c>
       <c r="G84" s="17" t="inlineStr">
         <is>
-          <t>No assessment/education subsystem in the prototype.</t>
+          <t>Competency = predicate tag.</t>
         </is>
       </c>
       <c r="H84" s="17" t="inlineStr"/>
@@ -4289,20 +4325,24 @@
           <t>6. Assessment / Education</t>
         </is>
       </c>
-      <c r="D86" s="21" t="inlineStr">
-        <is>
-          <t>Missing</t>
-        </is>
-      </c>
-      <c r="E86" s="22" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="F86" s="17" t="inlineStr"/>
+      <c r="D86" s="23" t="inlineStr">
+        <is>
+          <t>Included</t>
+        </is>
+      </c>
+      <c r="E86" s="24" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F86" s="17" t="inlineStr">
+        <is>
+          <t>qb_assess._difficulty</t>
+        </is>
+      </c>
       <c r="G86" s="17" t="inlineStr">
         <is>
-          <t>No assessment/education subsystem in the prototype.</t>
+          <t>Difficulty estimation.</t>
         </is>
       </c>
       <c r="H86" s="17" t="inlineStr"/>
@@ -4385,20 +4425,24 @@
           <t>6. Assessment / Education</t>
         </is>
       </c>
-      <c r="D89" s="21" t="inlineStr">
-        <is>
-          <t>Missing</t>
-        </is>
-      </c>
-      <c r="E89" s="22" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="F89" s="17" t="inlineStr"/>
+      <c r="D89" s="23" t="inlineStr">
+        <is>
+          <t>Included</t>
+        </is>
+      </c>
+      <c r="E89" s="24" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F89" s="17" t="inlineStr">
+        <is>
+          <t>qb_assess (provenance)</t>
+        </is>
+      </c>
       <c r="G89" s="17" t="inlineStr">
         <is>
-          <t>No assessment/education subsystem in the prototype.</t>
+          <t>Item provenance carried from Fact Units.</t>
         </is>
       </c>
       <c r="H89" s="17" t="inlineStr"/>
@@ -4417,20 +4461,24 @@
           <t>6. Assessment / Education</t>
         </is>
       </c>
-      <c r="D90" s="21" t="inlineStr">
-        <is>
-          <t>Missing</t>
-        </is>
-      </c>
-      <c r="E90" s="22" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="F90" s="17" t="inlineStr"/>
+      <c r="D90" s="23" t="inlineStr">
+        <is>
+          <t>Included</t>
+        </is>
+      </c>
+      <c r="E90" s="24" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F90" s="17" t="inlineStr">
+        <is>
+          <t>qb_assess.items_from_triples</t>
+        </is>
+      </c>
       <c r="G90" s="17" t="inlineStr">
         <is>
-          <t>No assessment/education subsystem in the prototype.</t>
+          <t>FU-linked item generator.</t>
         </is>
       </c>
       <c r="H90" s="17" t="inlineStr"/>
@@ -4673,20 +4721,24 @@
           <t>7. Licensing &amp; Rights</t>
         </is>
       </c>
-      <c r="D98" s="21" t="inlineStr">
-        <is>
-          <t>Missing</t>
-        </is>
-      </c>
-      <c r="E98" s="22" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="F98" s="17" t="inlineStr"/>
+      <c r="D98" s="23" t="inlineStr">
+        <is>
+          <t>Included</t>
+        </is>
+      </c>
+      <c r="E98" s="24" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F98" s="17" t="inlineStr">
+        <is>
+          <t>qb_rights (registry)</t>
+        </is>
+      </c>
       <c r="G98" s="17" t="inlineStr">
         <is>
-          <t>No licensing/rights subsystem in the prototype.</t>
+          <t>License registry.</t>
         </is>
       </c>
       <c r="H98" s="17" t="inlineStr"/>
@@ -4705,20 +4757,24 @@
           <t>7. Licensing &amp; Rights</t>
         </is>
       </c>
-      <c r="D99" s="21" t="inlineStr">
-        <is>
-          <t>Missing</t>
-        </is>
-      </c>
-      <c r="E99" s="22" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="F99" s="17" t="inlineStr"/>
+      <c r="D99" s="23" t="inlineStr">
+        <is>
+          <t>Included</t>
+        </is>
+      </c>
+      <c r="E99" s="24" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F99" s="17" t="inlineStr">
+        <is>
+          <t>qb_rights.check</t>
+        </is>
+      </c>
       <c r="G99" s="17" t="inlineStr">
         <is>
-          <t>No licensing/rights subsystem in the prototype.</t>
+          <t>Rights enforcement (allow/deny + reasons).</t>
         </is>
       </c>
       <c r="H99" s="17" t="inlineStr"/>
@@ -4737,20 +4793,24 @@
           <t>7. Licensing &amp; Rights</t>
         </is>
       </c>
-      <c r="D100" s="21" t="inlineStr">
-        <is>
-          <t>Missing</t>
-        </is>
-      </c>
-      <c r="E100" s="22" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="F100" s="17" t="inlineStr"/>
+      <c r="D100" s="23" t="inlineStr">
+        <is>
+          <t>Included</t>
+        </is>
+      </c>
+      <c r="E100" s="24" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F100" s="17" t="inlineStr">
+        <is>
+          <t>qb_rights (territories)</t>
+        </is>
+      </c>
       <c r="G100" s="17" t="inlineStr">
         <is>
-          <t>No licensing/rights subsystem in the prototype.</t>
+          <t>Territorial restrictions.</t>
         </is>
       </c>
       <c r="H100" s="17" t="inlineStr"/>
@@ -4769,20 +4829,24 @@
           <t>7. Licensing &amp; Rights</t>
         </is>
       </c>
-      <c r="D101" s="21" t="inlineStr">
-        <is>
-          <t>Missing</t>
-        </is>
-      </c>
-      <c r="E101" s="22" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="F101" s="17" t="inlineStr"/>
+      <c r="D101" s="23" t="inlineStr">
+        <is>
+          <t>Included</t>
+        </is>
+      </c>
+      <c r="E101" s="24" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F101" s="17" t="inlineStr">
+        <is>
+          <t>qb_rights (editions)</t>
+        </is>
+      </c>
       <c r="G101" s="17" t="inlineStr">
         <is>
-          <t>No licensing/rights subsystem in the prototype.</t>
+          <t>Edition restrictions.</t>
         </is>
       </c>
       <c r="H101" s="17" t="inlineStr"/>
@@ -4897,20 +4961,24 @@
           <t>7. Licensing &amp; Rights</t>
         </is>
       </c>
-      <c r="D105" s="21" t="inlineStr">
-        <is>
-          <t>Missing</t>
-        </is>
-      </c>
-      <c r="E105" s="22" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="F105" s="17" t="inlineStr"/>
+      <c r="D105" s="23" t="inlineStr">
+        <is>
+          <t>Included</t>
+        </is>
+      </c>
+      <c r="E105" s="24" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F105" s="17" t="inlineStr">
+        <is>
+          <t>qb_rights (expires)</t>
+        </is>
+      </c>
       <c r="G105" s="17" t="inlineStr">
         <is>
-          <t>No licensing/rights subsystem in the prototype.</t>
+          <t>License expiration handling.</t>
         </is>
       </c>
       <c r="H105" s="17" t="inlineStr"/>
@@ -4993,20 +5061,24 @@
           <t>7. Licensing &amp; Rights</t>
         </is>
       </c>
-      <c r="D108" s="21" t="inlineStr">
-        <is>
-          <t>Missing</t>
-        </is>
-      </c>
-      <c r="E108" s="22" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="F108" s="17" t="inlineStr"/>
+      <c r="D108" s="23" t="inlineStr">
+        <is>
+          <t>Included</t>
+        </is>
+      </c>
+      <c r="E108" s="24" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F108" s="17" t="inlineStr">
+        <is>
+          <t>qb_rights.check (scope)</t>
+        </is>
+      </c>
       <c r="G108" s="17" t="inlineStr">
         <is>
-          <t>No licensing/rights subsystem in the prototype.</t>
+          <t>License scope resolver.</t>
         </is>
       </c>
       <c r="H108" s="17" t="inlineStr"/>
@@ -5121,20 +5193,24 @@
           <t>8. NFT / Blockchain</t>
         </is>
       </c>
-      <c r="D112" s="21" t="inlineStr">
-        <is>
-          <t>Missing</t>
-        </is>
-      </c>
-      <c r="E112" s="22" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="F112" s="17" t="inlineStr"/>
+      <c r="D112" s="19" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="E112" s="20" t="inlineStr">
+        <is>
+          <t>~</t>
+        </is>
+      </c>
+      <c r="F112" s="17" t="inlineStr">
+        <is>
+          <t>qb_integrity (hash-chain ledger)</t>
+        </is>
+      </c>
       <c r="G112" s="17" t="inlineStr">
         <is>
-          <t>No NFT/blockchain minting in the prototype (provenance is SHA-256 Fact Units, not on-chain).</t>
+          <t>Local tamper-evident provenance; NOT on-chain NFT.</t>
         </is>
       </c>
       <c r="H112" s="17" t="inlineStr"/>
@@ -5185,20 +5261,24 @@
           <t>8. NFT / Blockchain</t>
         </is>
       </c>
-      <c r="D114" s="21" t="inlineStr">
-        <is>
-          <t>Missing</t>
-        </is>
-      </c>
-      <c r="E114" s="22" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="F114" s="17" t="inlineStr"/>
+      <c r="D114" s="23" t="inlineStr">
+        <is>
+          <t>Included</t>
+        </is>
+      </c>
+      <c r="E114" s="24" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F114" s="17" t="inlineStr">
+        <is>
+          <t>qb_integrity.lineage</t>
+        </is>
+      </c>
       <c r="G114" s="17" t="inlineStr">
         <is>
-          <t>No NFT/blockchain minting in the prototype (provenance is SHA-256 Fact Units, not on-chain).</t>
+          <t>Lineage chain manager (local hash chain).</t>
         </is>
       </c>
       <c r="H114" s="17" t="inlineStr"/>
@@ -5217,20 +5297,24 @@
           <t>8. NFT / Blockchain</t>
         </is>
       </c>
-      <c r="D115" s="21" t="inlineStr">
-        <is>
-          <t>Missing</t>
-        </is>
-      </c>
-      <c r="E115" s="22" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="F115" s="17" t="inlineStr"/>
+      <c r="D115" s="23" t="inlineStr">
+        <is>
+          <t>Included</t>
+        </is>
+      </c>
+      <c r="E115" s="24" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F115" s="17" t="inlineStr">
+        <is>
+          <t>qb_integrity.verify_chain</t>
+        </is>
+      </c>
       <c r="G115" s="17" t="inlineStr">
         <is>
-          <t>No NFT/blockchain minting in the prototype (provenance is SHA-256 Fact Units, not on-chain).</t>
+          <t>Ownership/integrity verification (local).</t>
         </is>
       </c>
       <c r="H115" s="17" t="inlineStr"/>
@@ -5669,20 +5753,24 @@
           <t>9. Reader Experience</t>
         </is>
       </c>
-      <c r="D129" s="21" t="inlineStr">
-        <is>
-          <t>Missing</t>
-        </is>
-      </c>
-      <c r="E129" s="22" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="F129" s="17" t="inlineStr"/>
+      <c r="D129" s="23" t="inlineStr">
+        <is>
+          <t>Included</t>
+        </is>
+      </c>
+      <c r="E129" s="24" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F129" s="17" t="inlineStr">
+        <is>
+          <t>qb_assess.study_guide</t>
+        </is>
+      </c>
       <c r="G129" s="17" t="inlineStr">
         <is>
-          <t>No reader-experience subsystem in the prototype.</t>
+          <t>Study-guide generator.</t>
         </is>
       </c>
       <c r="H129" s="17" t="inlineStr"/>
@@ -6709,24 +6797,24 @@
           <t>12. Response Generation</t>
         </is>
       </c>
-      <c r="D161" s="19" t="inlineStr">
-        <is>
-          <t>Partial</t>
-        </is>
-      </c>
-      <c r="E161" s="20" t="inlineStr">
-        <is>
-          <t>~</t>
+      <c r="D161" s="23" t="inlineStr">
+        <is>
+          <t>Included</t>
+        </is>
+      </c>
+      <c r="E161" s="24" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="F161" s="17" t="inlineStr">
         <is>
-          <t>qb_chat.retrieve (ranking)</t>
+          <t>qb_query.rank_evidence</t>
         </is>
       </c>
       <c r="G161" s="17" t="inlineStr">
         <is>
-          <t>Retrieved evidence is ranked; no dedicated ranking engine.</t>
+          <t>Lexical-overlap evidence ranking.</t>
         </is>
       </c>
       <c r="H161" s="17" t="inlineStr"/>
@@ -6745,24 +6833,24 @@
           <t>12. Response Generation</t>
         </is>
       </c>
-      <c r="D162" s="19" t="inlineStr">
-        <is>
-          <t>Partial</t>
-        </is>
-      </c>
-      <c r="E162" s="20" t="inlineStr">
-        <is>
-          <t>~</t>
+      <c r="D162" s="23" t="inlineStr">
+        <is>
+          <t>Included</t>
+        </is>
+      </c>
+      <c r="E162" s="24" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="F162" s="17" t="inlineStr">
         <is>
-          <t>qb_chat.compose/check</t>
+          <t>qb_query.rank_evidence (coherence)</t>
         </is>
       </c>
       <c r="G162" s="17" t="inlineStr">
         <is>
-          <t>Coherence check exists in compose/check.</t>
+          <t>Coherence flag on ranked evidence.</t>
         </is>
       </c>
       <c r="H162" s="17" t="inlineStr"/>
@@ -6817,24 +6905,24 @@
           <t>12. Response Generation</t>
         </is>
       </c>
-      <c r="D164" s="19" t="inlineStr">
-        <is>
-          <t>Partial</t>
-        </is>
-      </c>
-      <c r="E164" s="20" t="inlineStr">
-        <is>
-          <t>~</t>
+      <c r="D164" s="23" t="inlineStr">
+        <is>
+          <t>Included</t>
+        </is>
+      </c>
+      <c r="E164" s="24" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="F164" s="17" t="inlineStr">
         <is>
-          <t>qb_chat</t>
+          <t>qb_rights.redact</t>
         </is>
       </c>
       <c r="G164" s="17" t="inlineStr">
         <is>
-          <t>Partially realized by the chat answer pipeline.</t>
+          <t>Rights-aware redaction.</t>
         </is>
       </c>
       <c r="H164" s="17" t="inlineStr"/>
@@ -7317,20 +7405,24 @@
           <t>14. Deployment &amp; Integration</t>
         </is>
       </c>
-      <c r="D178" s="21" t="inlineStr">
-        <is>
-          <t>Missing</t>
-        </is>
-      </c>
-      <c r="E178" s="22" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="F178" s="17" t="inlineStr"/>
+      <c r="D178" s="23" t="inlineStr">
+        <is>
+          <t>Included</t>
+        </is>
+      </c>
+      <c r="E178" s="24" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F178" s="17" t="inlineStr">
+        <is>
+          <t>/api/webhooks</t>
+        </is>
+      </c>
       <c r="G178" s="17" t="inlineStr">
         <is>
-          <t>No webhooks/event-subscription system.</t>
+          <t>Webhook registry (register/list/clear).</t>
         </is>
       </c>
       <c r="H178" s="17" t="inlineStr"/>
@@ -8105,24 +8197,24 @@
           <t>17. LIL Identity / Voiceprint</t>
         </is>
       </c>
-      <c r="D200" s="19" t="inlineStr">
-        <is>
-          <t>Partial</t>
-        </is>
-      </c>
-      <c r="E200" s="20" t="inlineStr">
-        <is>
-          <t>~</t>
+      <c r="D200" s="23" t="inlineStr">
+        <is>
+          <t>Included</t>
+        </is>
+      </c>
+      <c r="E200" s="24" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="F200" s="17" t="inlineStr">
         <is>
-          <t>voice.html (Voice Lab)</t>
+          <t>qb_lil (enroll/match)</t>
         </is>
       </c>
       <c r="G200" s="17" t="inlineStr">
         <is>
-          <t>Voiceprint record/profile/match exists as a browser demo; no engine backend or persistent identity store.</t>
+          <t>Voiceprint engine backend (deterministic, consent-gated).</t>
         </is>
       </c>
       <c r="H200" s="17" t="inlineStr"/>
@@ -8141,24 +8233,24 @@
           <t>17. LIL Identity / Voiceprint</t>
         </is>
       </c>
-      <c r="D201" s="21" t="inlineStr">
-        <is>
-          <t>Missing</t>
-        </is>
-      </c>
-      <c r="E201" s="22" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D201" s="19" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="E201" s="20" t="inlineStr">
+        <is>
+          <t>~</t>
         </is>
       </c>
       <c r="F201" s="17" t="inlineStr">
         <is>
-          <t>voice.html</t>
+          <t>qb_lil (identity fields)</t>
         </is>
       </c>
       <c r="G201" s="17" t="inlineStr">
         <is>
-          <t>Design only / browser demo; no engine backend.</t>
+          <t>Links name/email/venue; full FU identity graph pending.</t>
         </is>
       </c>
       <c r="H201" s="17" t="inlineStr"/>
@@ -8177,24 +8269,24 @@
           <t>17. LIL Identity / Voiceprint</t>
         </is>
       </c>
-      <c r="D202" s="19" t="inlineStr">
-        <is>
-          <t>Partial</t>
-        </is>
-      </c>
-      <c r="E202" s="20" t="inlineStr">
-        <is>
-          <t>~</t>
+      <c r="D202" s="23" t="inlineStr">
+        <is>
+          <t>Included</t>
+        </is>
+      </c>
+      <c r="E202" s="24" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="F202" s="17" t="inlineStr">
         <is>
-          <t>voice.html consent + qb_language custom-voice consent gate</t>
+          <t>qb_lil + consent gate</t>
         </is>
       </c>
       <c r="G202" s="17" t="inlineStr">
         <is>
-          <t>Trust/consent gating is present in UI and for voice cloning; no identity-assertion engine.</t>
+          <t>Trust/consent-gated identity assertion (attributed).</t>
         </is>
       </c>
       <c r="H202" s="17" t="inlineStr"/>
@@ -8213,24 +8305,24 @@
           <t>17. LIL Identity / Voiceprint</t>
         </is>
       </c>
-      <c r="D203" s="21" t="inlineStr">
-        <is>
-          <t>Missing</t>
-        </is>
-      </c>
-      <c r="E203" s="22" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D203" s="19" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="E203" s="20" t="inlineStr">
+        <is>
+          <t>~</t>
         </is>
       </c>
       <c r="F203" s="17" t="inlineStr">
         <is>
-          <t>voice.html</t>
+          <t>qb_lil.authenticate</t>
         </is>
       </c>
       <c r="G203" s="17" t="inlineStr">
         <is>
-          <t>Design only / browser demo; no engine backend.</t>
+          <t>Voice auth built; anti-spoofing not implemented (labelled).</t>
         </is>
       </c>
       <c r="H203" s="17" t="inlineStr"/>
@@ -8249,24 +8341,24 @@
           <t>17. LIL Identity / Voiceprint</t>
         </is>
       </c>
-      <c r="D204" s="19" t="inlineStr">
-        <is>
-          <t>Partial</t>
-        </is>
-      </c>
-      <c r="E204" s="20" t="inlineStr">
-        <is>
-          <t>~</t>
+      <c r="D204" s="23" t="inlineStr">
+        <is>
+          <t>Included</t>
+        </is>
+      </c>
+      <c r="E204" s="24" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="F204" s="17" t="inlineStr">
         <is>
-          <t>voice.html vp-consent, qb_language.google_build_custom_voice (consent gate)</t>
+          <t xml:space="preserve">qb_lil (consent) </t>
         </is>
       </c>
       <c r="G204" s="17" t="inlineStr">
         <is>
-          <t>Consent gate enforced for voiceprints (UI) and voice cloning (engine).</t>
+          <t>Consent gate + local biometric privacy.</t>
         </is>
       </c>
       <c r="H204" s="17" t="inlineStr"/>
@@ -8285,20 +8377,24 @@
           <t>18. UIAS Integrity Audit</t>
         </is>
       </c>
-      <c r="D205" s="21" t="inlineStr">
-        <is>
-          <t>Missing</t>
-        </is>
-      </c>
-      <c r="E205" s="22" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="F205" s="17" t="inlineStr"/>
+      <c r="D205" s="23" t="inlineStr">
+        <is>
+          <t>Included</t>
+        </is>
+      </c>
+      <c r="E205" s="24" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F205" s="17" t="inlineStr">
+        <is>
+          <t>qb_integrity.seal</t>
+        </is>
+      </c>
       <c r="G205" s="17" t="inlineStr">
         <is>
-          <t>Design only; no prototype implementation.</t>
+          <t>Pre-dispute timestamped seal (seal = Fact Unit).</t>
         </is>
       </c>
       <c r="H205" s="17" t="inlineStr"/>
@@ -8317,20 +8413,24 @@
           <t>18. UIAS Integrity Audit</t>
         </is>
       </c>
-      <c r="D206" s="21" t="inlineStr">
-        <is>
-          <t>Missing</t>
-        </is>
-      </c>
-      <c r="E206" s="22" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="F206" s="17" t="inlineStr"/>
+      <c r="D206" s="23" t="inlineStr">
+        <is>
+          <t>Included</t>
+        </is>
+      </c>
+      <c r="E206" s="24" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F206" s="17" t="inlineStr">
+        <is>
+          <t>qb_integrity.similarity</t>
+        </is>
+      </c>
       <c r="G206" s="17" t="inlineStr">
         <is>
-          <t>Design only; no prototype implementation.</t>
+          <t>Cross-submission k-shingle Jaccard similarity.</t>
         </is>
       </c>
       <c r="H206" s="17" t="inlineStr"/>
@@ -8349,20 +8449,24 @@
           <t>18. UIAS Integrity Audit</t>
         </is>
       </c>
-      <c r="D207" s="21" t="inlineStr">
-        <is>
-          <t>Missing</t>
-        </is>
-      </c>
-      <c r="E207" s="22" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="F207" s="17" t="inlineStr"/>
+      <c r="D207" s="23" t="inlineStr">
+        <is>
+          <t>Included</t>
+        </is>
+      </c>
+      <c r="E207" s="24" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F207" s="17" t="inlineStr">
+        <is>
+          <t>qb_integrity.proof_package</t>
+        </is>
+      </c>
       <c r="G207" s="17" t="inlineStr">
         <is>
-          <t>Design only; no prototype implementation.</t>
+          <t>HMAC-signed proof package (local).</t>
         </is>
       </c>
       <c r="H207" s="17" t="inlineStr"/>
@@ -8477,24 +8581,24 @@
           <t>19. PIL Interpretation</t>
         </is>
       </c>
-      <c r="D211" s="19" t="inlineStr">
-        <is>
-          <t>Partial</t>
-        </is>
-      </c>
-      <c r="E211" s="20" t="inlineStr">
-        <is>
-          <t>~</t>
+      <c r="D211" s="23" t="inlineStr">
+        <is>
+          <t>Included</t>
+        </is>
+      </c>
+      <c r="E211" s="24" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="F211" s="17" t="inlineStr">
         <is>
-          <t>voice.html (tone/arousal/pacing demo)</t>
+          <t>qb_pil.analyze</t>
         </is>
       </c>
       <c r="G211" s="17" t="inlineStr">
         <is>
-          <t>Paralinguistic acoustic estimates exist as a browser demo; no engine backend.</t>
+          <t>Paralinguistic measured estimates backend.</t>
         </is>
       </c>
       <c r="H211" s="17" t="inlineStr"/>
@@ -8513,20 +8617,24 @@
           <t>19. PIL Interpretation</t>
         </is>
       </c>
-      <c r="D212" s="21" t="inlineStr">
-        <is>
-          <t>Missing</t>
-        </is>
-      </c>
-      <c r="E212" s="22" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="F212" s="17" t="inlineStr"/>
+      <c r="D212" s="23" t="inlineStr">
+        <is>
+          <t>Included</t>
+        </is>
+      </c>
+      <c r="E212" s="24" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F212" s="17" t="inlineStr">
+        <is>
+          <t>qb_pil.pragmatics</t>
+        </is>
+      </c>
       <c r="G212" s="17" t="inlineStr">
         <is>
-          <t>Design only; no prototype implementation.</t>
+          <t>Pragmatic framing (sourced cues).</t>
         </is>
       </c>
       <c r="H212" s="17" t="inlineStr"/>
@@ -8577,20 +8685,24 @@
           <t>19. PIL Interpretation</t>
         </is>
       </c>
-      <c r="D214" s="21" t="inlineStr">
-        <is>
-          <t>Missing</t>
-        </is>
-      </c>
-      <c r="E214" s="22" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="F214" s="17" t="inlineStr"/>
+      <c r="D214" s="23" t="inlineStr">
+        <is>
+          <t>Included</t>
+        </is>
+      </c>
+      <c r="E214" s="24" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F214" s="17" t="inlineStr">
+        <is>
+          <t>qb_pil.interpret_query + qb_query</t>
+        </is>
+      </c>
       <c r="G214" s="17" t="inlineStr">
         <is>
-          <t>Design only; no prototype implementation.</t>
+          <t>Query interpretation front stage.</t>
         </is>
       </c>
       <c r="H214" s="17" t="inlineStr"/>
@@ -8920,11 +9032,11 @@
         <v>1</v>
       </c>
       <c r="C8" s="26" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="D8" s="27" t="inlineStr">
         <is>
-          <t>59, 60, 61, 63, 64, 65, 66</t>
+          <t>64, 66</t>
         </is>
       </c>
     </row>
@@ -8935,14 +9047,14 @@
         </is>
       </c>
       <c r="B9" s="26" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="C9" s="26" t="n">
         <v>0</v>
       </c>
       <c r="D9" s="27" t="inlineStr">
         <is>
-          <t>68, 69, 70, 71, 72, 73, 74, 75, 76, 77, 78, 79, 80</t>
+          <t>74, 75, 76, 77, 78, 79, 80</t>
         </is>
       </c>
     </row>
@@ -8953,14 +9065,14 @@
         </is>
       </c>
       <c r="B10" s="26" t="n">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="C10" s="26" t="n">
         <v>0</v>
       </c>
       <c r="D10" s="27" t="inlineStr">
         <is>
-          <t>81, 82, 83, 84, 85, 86, 87, 88, 89, 90, 91, 92, 93, 94, 95, 96</t>
+          <t>84, 86, 87, 90, 91, 92, 93, 94, 95, 96</t>
         </is>
       </c>
     </row>
@@ -8971,14 +9083,14 @@
         </is>
       </c>
       <c r="B11" s="26" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="C11" s="26" t="n">
         <v>0</v>
       </c>
       <c r="D11" s="27" t="inlineStr">
         <is>
-          <t>97, 98, 99, 100, 101, 102, 103, 104, 105, 106, 107, 108</t>
+          <t>101, 102, 103, 105, 106, 108</t>
         </is>
       </c>
     </row>
@@ -8989,14 +9101,14 @@
         </is>
       </c>
       <c r="B12" s="26" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="C12" s="26" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D12" s="27" t="inlineStr">
         <is>
-          <t>109, 110, 111, 112, 113, 114, 115, 116, 117, 118</t>
+          <t>109, 110, 111, 112, 115, 116, 117, 118</t>
         </is>
       </c>
     </row>
@@ -9007,14 +9119,14 @@
         </is>
       </c>
       <c r="B13" s="26" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C13" s="26" t="n">
         <v>1</v>
       </c>
       <c r="D13" s="27" t="inlineStr">
         <is>
-          <t>119, 120, 121, 122, 123, 124, 125, 126, 127, 128, 129, 130</t>
+          <t>119, 120, 121, 122, 123, 124, 125, 126, 127, 129, 130</t>
         </is>
       </c>
     </row>
@@ -9064,11 +9176,11 @@
         <v>1</v>
       </c>
       <c r="C16" s="26" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="D16" s="27" t="inlineStr">
         <is>
-          <t>159, 160, 161, 162, 163, 164, 165</t>
+          <t>159, 162, 164, 165</t>
         </is>
       </c>
     </row>
@@ -9097,14 +9209,14 @@
         </is>
       </c>
       <c r="B18" s="26" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C18" s="26" t="n">
         <v>4</v>
       </c>
       <c r="D18" s="27" t="inlineStr">
         <is>
-          <t>173, 174, 175, 176, 177</t>
+          <t>173, 174, 175, 176</t>
         </is>
       </c>
     </row>
@@ -9151,14 +9263,14 @@
         </is>
       </c>
       <c r="B21" s="26" t="n">
+        <v>0</v>
+      </c>
+      <c r="C21" s="26" t="n">
         <v>2</v>
       </c>
-      <c r="C21" s="26" t="n">
-        <v>3</v>
-      </c>
       <c r="D21" s="27" t="inlineStr">
         <is>
-          <t>199, 200, 201, 202, 203</t>
+          <t>200, 202</t>
         </is>
       </c>
     </row>
@@ -9169,14 +9281,14 @@
         </is>
       </c>
       <c r="B22" s="26" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="C22" s="26" t="n">
         <v>0</v>
       </c>
       <c r="D22" s="27" t="inlineStr">
         <is>
-          <t>204, 205, 206, 207, 208, 209</t>
+          <t>207, 208, 209</t>
         </is>
       </c>
     </row>
@@ -9187,14 +9299,14 @@
         </is>
       </c>
       <c r="B23" s="26" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C23" s="26" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D23" s="27" t="inlineStr">
         <is>
-          <t>210, 211, 212, 213</t>
+          <t>212</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
v9.56: sync canon for Education + SaaS; package build
- Registry: added [227]-[231] (Learner/Reader, Educator analytics, Collaboration,
  SaaS admin, Education covenant); count → 235; Registry.docx regenerated.
- Bible: amendment "Education & Multi-Tenant SaaS (2026-10-02)"; Bible.docx regenerated.
- Audit regenerated: Included 75→100, Missing 120→96 (226 enumerated features);
  Excel + checkbox Word refreshed.
- Sync report regenerated (v9.56, 34/34 live).
- Page versions unified to v9.56; home links Learn/Educator/Collaborate/Admin.
- Repackaged QueryBook-v9.56-2026-10-02.zip (407 files, no secrets).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019szkZU7hLaBcGBEqVSVWY6
</commit_message>
<xml_diff>
--- a/docs/QueryBook-Prototype-Registry-Audit.xlsx
+++ b/docs/QueryBook-Prototype-Registry-Audit.xlsx
@@ -576,7 +576,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Prototype: QueryBook v9.55  ·  Registry: 219 enumerated features  ·  Date: 2026-10-02</t>
+          <t>Prototype: QueryBook v9.56  ·  Registry: 219 enumerated features  ·  Date: 2026-10-02</t>
         </is>
       </c>
     </row>
@@ -611,10 +611,10 @@
         </is>
       </c>
       <c r="B6" s="6" t="n">
-        <v>75</v>
+        <v>100</v>
       </c>
       <c r="C6" s="6" t="n">
-        <v>33.2</v>
+        <v>44.2</v>
       </c>
     </row>
     <row r="7">
@@ -624,10 +624,10 @@
         </is>
       </c>
       <c r="B7" s="8" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C7" s="8" t="n">
-        <v>13.7</v>
+        <v>13.3</v>
       </c>
     </row>
     <row r="8">
@@ -637,10 +637,10 @@
         </is>
       </c>
       <c r="B8" s="10" t="n">
-        <v>120</v>
+        <v>96</v>
       </c>
       <c r="C8" s="10" t="n">
-        <v>53.1</v>
+        <v>42.5</v>
       </c>
     </row>
     <row r="9">
@@ -659,7 +659,7 @@
     <row r="11">
       <c r="A11" s="12" t="inlineStr">
         <is>
-          <t>Reading: the prototype fully supports 75 features and partially supports 31 (= 106 of 219, 47% touched); 120 are not present.</t>
+          <t>Reading: the prototype fully supports 100 features and partially supports 30 (= 130 of 219, 58% touched); 96 are not present.</t>
         </is>
       </c>
     </row>
@@ -856,13 +856,13 @@
         </is>
       </c>
       <c r="B23" s="13" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="C23" s="13" t="n">
         <v>1</v>
       </c>
       <c r="D23" s="13" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="E23" s="13" t="n">
         <v>12</v>
@@ -875,13 +875,13 @@
         </is>
       </c>
       <c r="B24" s="13" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="C24" s="13" t="n">
         <v>0</v>
       </c>
       <c r="D24" s="13" t="n">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="E24" s="13" t="n">
         <v>15</v>
@@ -894,13 +894,13 @@
         </is>
       </c>
       <c r="B25" s="13" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="C25" s="13" t="n">
         <v>0</v>
       </c>
       <c r="D25" s="13" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="E25" s="13" t="n">
         <v>10</v>
@@ -935,10 +935,10 @@
         <v>0</v>
       </c>
       <c r="C27" s="13" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D27" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E27" s="13" t="n">
         <v>7</v>
@@ -951,10 +951,10 @@
         </is>
       </c>
       <c r="B28" s="13" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C28" s="13" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D28" s="13" t="n">
         <v>0</v>
@@ -1103,13 +1103,13 @@
         </is>
       </c>
       <c r="B36" s="11" t="n">
-        <v>75</v>
+        <v>100</v>
       </c>
       <c r="C36" s="11" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D36" s="11" t="n">
-        <v>120</v>
+        <v>96</v>
       </c>
       <c r="E36" s="11" t="n">
         <v>226</v>
@@ -5480,20 +5480,24 @@
           <t>9. Reader Experience</t>
         </is>
       </c>
-      <c r="D120" s="21" t="inlineStr">
-        <is>
-          <t>Missing</t>
-        </is>
-      </c>
-      <c r="E120" s="22" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="F120" s="17" t="inlineStr"/>
+      <c r="D120" s="23" t="inlineStr">
+        <is>
+          <t>Included</t>
+        </is>
+      </c>
+      <c r="E120" s="24" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F120" s="17" t="inlineStr">
+        <is>
+          <t>qb_education.generate_lesson</t>
+        </is>
+      </c>
       <c r="G120" s="17" t="inlineStr">
         <is>
-          <t>No reader-experience subsystem in the prototype.</t>
+          <t>Adaptive lesson path from Fact Units.</t>
         </is>
       </c>
       <c r="H120" s="17" t="inlineStr"/>
@@ -5548,20 +5552,24 @@
           <t>9. Reader Experience</t>
         </is>
       </c>
-      <c r="D122" s="21" t="inlineStr">
-        <is>
-          <t>Missing</t>
-        </is>
-      </c>
-      <c r="E122" s="22" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="F122" s="17" t="inlineStr"/>
+      <c r="D122" s="23" t="inlineStr">
+        <is>
+          <t>Included</t>
+        </is>
+      </c>
+      <c r="E122" s="24" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F122" s="17" t="inlineStr">
+        <is>
+          <t>qb_education (learner state)</t>
+        </is>
+      </c>
       <c r="G122" s="17" t="inlineStr">
         <is>
-          <t>No reader-experience subsystem in the prototype.</t>
+          <t>Reader state model (mastery/attempts).</t>
         </is>
       </c>
       <c r="H122" s="17" t="inlineStr"/>
@@ -5580,20 +5588,24 @@
           <t>9. Reader Experience</t>
         </is>
       </c>
-      <c r="D123" s="21" t="inlineStr">
-        <is>
-          <t>Missing</t>
-        </is>
-      </c>
-      <c r="E123" s="22" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="F123" s="17" t="inlineStr"/>
+      <c r="D123" s="23" t="inlineStr">
+        <is>
+          <t>Included</t>
+        </is>
+      </c>
+      <c r="E123" s="24" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F123" s="17" t="inlineStr">
+        <is>
+          <t>qb_education.learner_state</t>
+        </is>
+      </c>
       <c r="G123" s="17" t="inlineStr">
         <is>
-          <t>No reader-experience subsystem in the prototype.</t>
+          <t>Reader behavior analytics (engagement).</t>
         </is>
       </c>
       <c r="H123" s="17" t="inlineStr"/>
@@ -5612,20 +5624,24 @@
           <t>9. Reader Experience</t>
         </is>
       </c>
-      <c r="D124" s="21" t="inlineStr">
-        <is>
-          <t>Missing</t>
-        </is>
-      </c>
-      <c r="E124" s="22" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="F124" s="17" t="inlineStr"/>
+      <c r="D124" s="23" t="inlineStr">
+        <is>
+          <t>Included</t>
+        </is>
+      </c>
+      <c r="E124" s="24" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F124" s="17" t="inlineStr">
+        <is>
+          <t>qb_education (misconceptions)</t>
+        </is>
+      </c>
       <c r="G124" s="17" t="inlineStr">
         <is>
-          <t>No reader-experience subsystem in the prototype.</t>
+          <t>Misconception detection on wrong answers.</t>
         </is>
       </c>
       <c r="H124" s="17" t="inlineStr"/>
@@ -5644,20 +5660,24 @@
           <t>9. Reader Experience</t>
         </is>
       </c>
-      <c r="D125" s="21" t="inlineStr">
-        <is>
-          <t>Missing</t>
-        </is>
-      </c>
-      <c r="E125" s="22" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="F125" s="17" t="inlineStr"/>
+      <c r="D125" s="23" t="inlineStr">
+        <is>
+          <t>Included</t>
+        </is>
+      </c>
+      <c r="E125" s="24" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F125" s="17" t="inlineStr">
+        <is>
+          <t>qb_education (remediation)</t>
+        </is>
+      </c>
       <c r="G125" s="17" t="inlineStr">
         <is>
-          <t>No reader-experience subsystem in the prototype.</t>
+          <t>Remediation list from missed competencies.</t>
         </is>
       </c>
       <c r="H125" s="17" t="inlineStr"/>
@@ -5676,20 +5696,24 @@
           <t>9. Reader Experience</t>
         </is>
       </c>
-      <c r="D126" s="21" t="inlineStr">
-        <is>
-          <t>Missing</t>
-        </is>
-      </c>
-      <c r="E126" s="22" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="F126" s="17" t="inlineStr"/>
+      <c r="D126" s="23" t="inlineStr">
+        <is>
+          <t>Included</t>
+        </is>
+      </c>
+      <c r="E126" s="24" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F126" s="17" t="inlineStr">
+        <is>
+          <t>qb_education.learner_state</t>
+        </is>
+      </c>
       <c r="G126" s="17" t="inlineStr">
         <is>
-          <t>No reader-experience subsystem in the prototype.</t>
+          <t>Reader personalization (per-learner mastery).</t>
         </is>
       </c>
       <c r="H126" s="17" t="inlineStr"/>
@@ -5708,20 +5732,24 @@
           <t>9. Reader Experience</t>
         </is>
       </c>
-      <c r="D127" s="21" t="inlineStr">
-        <is>
-          <t>Missing</t>
-        </is>
-      </c>
-      <c r="E127" s="22" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="F127" s="17" t="inlineStr"/>
+      <c r="D127" s="23" t="inlineStr">
+        <is>
+          <t>Included</t>
+        </is>
+      </c>
+      <c r="E127" s="24" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F127" s="17" t="inlineStr">
+        <is>
+          <t>qb_ontology + /learn</t>
+        </is>
+      </c>
       <c r="G127" s="17" t="inlineStr">
         <is>
-          <t>No reader-experience subsystem in the prototype.</t>
+          <t>Concept map generator.</t>
         </is>
       </c>
       <c r="H127" s="17" t="inlineStr"/>
@@ -5784,7 +5812,7 @@
       </c>
       <c r="F129" s="17" t="inlineStr">
         <is>
-          <t>qb_assess.study_guide</t>
+          <t>qb_education.study_guide</t>
         </is>
       </c>
       <c r="G129" s="17" t="inlineStr">
@@ -5808,20 +5836,24 @@
           <t>9. Reader Experience</t>
         </is>
       </c>
-      <c r="D130" s="21" t="inlineStr">
-        <is>
-          <t>Missing</t>
-        </is>
-      </c>
-      <c r="E130" s="22" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="F130" s="17" t="inlineStr"/>
+      <c r="D130" s="23" t="inlineStr">
+        <is>
+          <t>Included</t>
+        </is>
+      </c>
+      <c r="E130" s="24" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F130" s="17" t="inlineStr">
+        <is>
+          <t>qb_education (engagement)</t>
+        </is>
+      </c>
       <c r="G130" s="17" t="inlineStr">
         <is>
-          <t>No reader-experience subsystem in the prototype.</t>
+          <t>Engagement scoring.</t>
         </is>
       </c>
       <c r="H130" s="17" t="inlineStr"/>
@@ -5840,20 +5872,24 @@
           <t>9. Reader Experience</t>
         </is>
       </c>
-      <c r="D131" s="21" t="inlineStr">
-        <is>
-          <t>Missing</t>
-        </is>
-      </c>
-      <c r="E131" s="22" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="F131" s="17" t="inlineStr"/>
+      <c r="D131" s="23" t="inlineStr">
+        <is>
+          <t>Included</t>
+        </is>
+      </c>
+      <c r="E131" s="24" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F131" s="17" t="inlineStr">
+        <is>
+          <t>qb_education (attempts)</t>
+        </is>
+      </c>
       <c r="G131" s="17" t="inlineStr">
         <is>
-          <t>No reader-experience subsystem in the prototype.</t>
+          <t>Reader session tracking.</t>
         </is>
       </c>
       <c r="H131" s="17" t="inlineStr"/>
@@ -5872,20 +5908,24 @@
           <t>10. Educator Analytics</t>
         </is>
       </c>
-      <c r="D132" s="21" t="inlineStr">
-        <is>
-          <t>Missing</t>
-        </is>
-      </c>
-      <c r="E132" s="22" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="F132" s="17" t="inlineStr"/>
+      <c r="D132" s="23" t="inlineStr">
+        <is>
+          <t>Included</t>
+        </is>
+      </c>
+      <c r="E132" s="24" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F132" s="17" t="inlineStr">
+        <is>
+          <t>/educator + qb_education.class_analytics</t>
+        </is>
+      </c>
       <c r="G132" s="17" t="inlineStr">
         <is>
-          <t>No educator analytics subsystem in the prototype.</t>
+          <t>Educator dashboard.</t>
         </is>
       </c>
       <c r="H132" s="17" t="inlineStr"/>
@@ -5904,20 +5944,24 @@
           <t>10. Educator Analytics</t>
         </is>
       </c>
-      <c r="D133" s="21" t="inlineStr">
-        <is>
-          <t>Missing</t>
-        </is>
-      </c>
-      <c r="E133" s="22" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="F133" s="17" t="inlineStr"/>
+      <c r="D133" s="23" t="inlineStr">
+        <is>
+          <t>Included</t>
+        </is>
+      </c>
+      <c r="E133" s="24" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F133" s="17" t="inlineStr">
+        <is>
+          <t>qb_education.class_analytics</t>
+        </is>
+      </c>
       <c r="G133" s="17" t="inlineStr">
         <is>
-          <t>No educator analytics subsystem in the prototype.</t>
+          <t>Class mastery aggregator.</t>
         </is>
       </c>
       <c r="H133" s="17" t="inlineStr"/>
@@ -5936,20 +5980,24 @@
           <t>10. Educator Analytics</t>
         </is>
       </c>
-      <c r="D134" s="21" t="inlineStr">
-        <is>
-          <t>Missing</t>
-        </is>
-      </c>
-      <c r="E134" s="22" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="F134" s="17" t="inlineStr"/>
+      <c r="D134" s="23" t="inlineStr">
+        <is>
+          <t>Included</t>
+        </is>
+      </c>
+      <c r="E134" s="24" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F134" s="17" t="inlineStr">
+        <is>
+          <t>qb_education (clusters)</t>
+        </is>
+      </c>
       <c r="G134" s="17" t="inlineStr">
         <is>
-          <t>No educator analytics subsystem in the prototype.</t>
+          <t>Misconception cluster.</t>
         </is>
       </c>
       <c r="H134" s="17" t="inlineStr"/>
@@ -5968,20 +6016,24 @@
           <t>10. Educator Analytics</t>
         </is>
       </c>
-      <c r="D135" s="21" t="inlineStr">
-        <is>
-          <t>Missing</t>
-        </is>
-      </c>
-      <c r="E135" s="22" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="F135" s="17" t="inlineStr"/>
+      <c r="D135" s="23" t="inlineStr">
+        <is>
+          <t>Included</t>
+        </is>
+      </c>
+      <c r="E135" s="24" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F135" s="17" t="inlineStr">
+        <is>
+          <t>qb_education (engagement)</t>
+        </is>
+      </c>
       <c r="G135" s="17" t="inlineStr">
         <is>
-          <t>No educator analytics subsystem in the prototype.</t>
+          <t>Engagement analytics.</t>
         </is>
       </c>
       <c r="H135" s="17" t="inlineStr"/>
@@ -6160,20 +6212,24 @@
           <t>10. Educator Analytics</t>
         </is>
       </c>
-      <c r="D141" s="21" t="inlineStr">
-        <is>
-          <t>Missing</t>
-        </is>
-      </c>
-      <c r="E141" s="22" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="F141" s="17" t="inlineStr"/>
+      <c r="D141" s="23" t="inlineStr">
+        <is>
+          <t>Included</t>
+        </is>
+      </c>
+      <c r="E141" s="24" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F141" s="17" t="inlineStr">
+        <is>
+          <t>qb_education (attempts)</t>
+        </is>
+      </c>
       <c r="G141" s="17" t="inlineStr">
         <is>
-          <t>No educator analytics subsystem in the prototype.</t>
+          <t>Class progress tracker.</t>
         </is>
       </c>
       <c r="H141" s="17" t="inlineStr"/>
@@ -6192,20 +6248,24 @@
           <t>10. Educator Analytics</t>
         </is>
       </c>
-      <c r="D142" s="21" t="inlineStr">
-        <is>
-          <t>Missing</t>
-        </is>
-      </c>
-      <c r="E142" s="22" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="F142" s="17" t="inlineStr"/>
+      <c r="D142" s="23" t="inlineStr">
+        <is>
+          <t>Included</t>
+        </is>
+      </c>
+      <c r="E142" s="24" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F142" s="17" t="inlineStr">
+        <is>
+          <t>qb_education (scores)</t>
+        </is>
+      </c>
       <c r="G142" s="17" t="inlineStr">
         <is>
-          <t>No educator analytics subsystem in the prototype.</t>
+          <t>Assignment performance.</t>
         </is>
       </c>
       <c r="H142" s="17" t="inlineStr"/>
@@ -6224,20 +6284,24 @@
           <t>10. Educator Analytics</t>
         </is>
       </c>
-      <c r="D143" s="21" t="inlineStr">
-        <is>
-          <t>Missing</t>
-        </is>
-      </c>
-      <c r="E143" s="22" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="F143" s="17" t="inlineStr"/>
+      <c r="D143" s="23" t="inlineStr">
+        <is>
+          <t>Included</t>
+        </is>
+      </c>
+      <c r="E143" s="24" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F143" s="17" t="inlineStr">
+        <is>
+          <t>qb_education.class_analytics (cohort)</t>
+        </is>
+      </c>
       <c r="G143" s="17" t="inlineStr">
         <is>
-          <t>No educator analytics subsystem in the prototype.</t>
+          <t>Cohort comparison.</t>
         </is>
       </c>
       <c r="H143" s="17" t="inlineStr"/>
@@ -6352,20 +6416,24 @@
           <t>11. Collaboration</t>
         </is>
       </c>
-      <c r="D147" s="21" t="inlineStr">
-        <is>
-          <t>Missing</t>
-        </is>
-      </c>
-      <c r="E147" s="22" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="F147" s="17" t="inlineStr"/>
+      <c r="D147" s="23" t="inlineStr">
+        <is>
+          <t>Included</t>
+        </is>
+      </c>
+      <c r="E147" s="24" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F147" s="17" t="inlineStr">
+        <is>
+          <t>qb_collab.add_annotation</t>
+        </is>
+      </c>
       <c r="G147" s="17" t="inlineStr">
         <is>
-          <t>No collaboration subsystem in the prototype.</t>
+          <t>Annotation engine.</t>
         </is>
       </c>
       <c r="H147" s="17" t="inlineStr"/>
@@ -6384,20 +6452,24 @@
           <t>11. Collaboration</t>
         </is>
       </c>
-      <c r="D148" s="21" t="inlineStr">
-        <is>
-          <t>Missing</t>
-        </is>
-      </c>
-      <c r="E148" s="22" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="F148" s="17" t="inlineStr"/>
+      <c r="D148" s="23" t="inlineStr">
+        <is>
+          <t>Included</t>
+        </is>
+      </c>
+      <c r="E148" s="24" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F148" s="17" t="inlineStr">
+        <is>
+          <t>qb_collab.post_thread</t>
+        </is>
+      </c>
       <c r="G148" s="17" t="inlineStr">
         <is>
-          <t>No collaboration subsystem in the prototype.</t>
+          <t>Threaded discussion.</t>
         </is>
       </c>
       <c r="H148" s="17" t="inlineStr"/>
@@ -6448,20 +6520,24 @@
           <t>11. Collaboration</t>
         </is>
       </c>
-      <c r="D150" s="21" t="inlineStr">
-        <is>
-          <t>Missing</t>
-        </is>
-      </c>
-      <c r="E150" s="22" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="F150" s="17" t="inlineStr"/>
+      <c r="D150" s="23" t="inlineStr">
+        <is>
+          <t>Included</t>
+        </is>
+      </c>
+      <c r="E150" s="24" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F150" s="17" t="inlineStr">
+        <is>
+          <t>qb_collab (seal)</t>
+        </is>
+      </c>
       <c r="G150" s="17" t="inlineStr">
         <is>
-          <t>No collaboration subsystem in the prototype.</t>
+          <t>Annotation provenance (sealed).</t>
         </is>
       </c>
       <c r="H150" s="17" t="inlineStr"/>
@@ -6480,20 +6556,24 @@
           <t>11. Collaboration</t>
         </is>
       </c>
-      <c r="D151" s="21" t="inlineStr">
-        <is>
-          <t>Missing</t>
-        </is>
-      </c>
-      <c r="E151" s="22" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="F151" s="17" t="inlineStr"/>
+      <c r="D151" s="23" t="inlineStr">
+        <is>
+          <t>Included</t>
+        </is>
+      </c>
+      <c r="E151" s="24" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F151" s="17" t="inlineStr">
+        <is>
+          <t>qb_collab (resources/tenant)</t>
+        </is>
+      </c>
       <c r="G151" s="17" t="inlineStr">
         <is>
-          <t>No collaboration subsystem in the prototype.</t>
+          <t>Group workspace.</t>
         </is>
       </c>
       <c r="H151" s="17" t="inlineStr"/>
@@ -6512,20 +6592,24 @@
           <t>11. Collaboration</t>
         </is>
       </c>
-      <c r="D152" s="21" t="inlineStr">
-        <is>
-          <t>Missing</t>
-        </is>
-      </c>
-      <c r="E152" s="22" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="F152" s="17" t="inlineStr"/>
+      <c r="D152" s="23" t="inlineStr">
+        <is>
+          <t>Included</t>
+        </is>
+      </c>
+      <c r="E152" s="24" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F152" s="17" t="inlineStr">
+        <is>
+          <t>qb_collab.add_resource</t>
+        </is>
+      </c>
       <c r="G152" s="17" t="inlineStr">
         <is>
-          <t>No collaboration subsystem in the prototype.</t>
+          <t>Shared resource manager.</t>
         </is>
       </c>
       <c r="H152" s="17" t="inlineStr"/>
@@ -6608,20 +6692,24 @@
           <t>11. Collaboration</t>
         </is>
       </c>
-      <c r="D155" s="21" t="inlineStr">
-        <is>
-          <t>Missing</t>
-        </is>
-      </c>
-      <c r="E155" s="22" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="F155" s="17" t="inlineStr"/>
+      <c r="D155" s="23" t="inlineStr">
+        <is>
+          <t>Included</t>
+        </is>
+      </c>
+      <c r="E155" s="24" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F155" s="17" t="inlineStr">
+        <is>
+          <t>qb_collab.activity</t>
+        </is>
+      </c>
       <c r="G155" s="17" t="inlineStr">
         <is>
-          <t>No collaboration subsystem in the prototype.</t>
+          <t>Collaboration activity feed.</t>
         </is>
       </c>
       <c r="H155" s="17" t="inlineStr"/>
@@ -6640,20 +6728,24 @@
           <t>11. Collaboration</t>
         </is>
       </c>
-      <c r="D156" s="21" t="inlineStr">
-        <is>
-          <t>Missing</t>
-        </is>
-      </c>
-      <c r="E156" s="22" t="inlineStr">
-        <is>
-          <t>✗</t>
-        </is>
-      </c>
-      <c r="F156" s="17" t="inlineStr"/>
+      <c r="D156" s="23" t="inlineStr">
+        <is>
+          <t>Included</t>
+        </is>
+      </c>
+      <c r="E156" s="24" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="F156" s="17" t="inlineStr">
+        <is>
+          <t>qb_collab (threads)</t>
+        </is>
+      </c>
       <c r="G156" s="17" t="inlineStr">
         <is>
-          <t>No collaboration subsystem in the prototype.</t>
+          <t>Collaboration session.</t>
         </is>
       </c>
       <c r="H156" s="17" t="inlineStr"/>
@@ -7208,24 +7300,24 @@
           <t>13. Analytics &amp; Quality</t>
         </is>
       </c>
-      <c r="D172" s="21" t="inlineStr">
-        <is>
-          <t>Missing</t>
-        </is>
-      </c>
-      <c r="E172" s="22" t="inlineStr">
-        <is>
-          <t>✗</t>
+      <c r="D172" s="19" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="E172" s="20" t="inlineStr">
+        <is>
+          <t>~</t>
         </is>
       </c>
       <c r="F172" s="17" t="inlineStr">
         <is>
-          <t>dashboard.html (ops only)</t>
+          <t>/educator dashboard</t>
         </is>
       </c>
       <c r="G172" s="17" t="inlineStr">
         <is>
-          <t>An ops console exists, but not a publisher analytics dashboard.</t>
+          <t>Educator dashboard exists; publisher analytics partial.</t>
         </is>
       </c>
       <c r="H172" s="17" t="inlineStr"/>
@@ -7280,24 +7372,24 @@
           <t>14. Deployment &amp; Integration</t>
         </is>
       </c>
-      <c r="D174" s="19" t="inlineStr">
-        <is>
-          <t>Partial</t>
-        </is>
-      </c>
-      <c r="E174" s="20" t="inlineStr">
-        <is>
-          <t>~</t>
+      <c r="D174" s="23" t="inlineStr">
+        <is>
+          <t>Included</t>
+        </is>
+      </c>
+      <c r="E174" s="24" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="F174" s="17" t="inlineStr">
         <is>
-          <t>QB_BIND env, START-*.command/.bat</t>
+          <t>qb_saas (plans/tenants)</t>
         </is>
       </c>
       <c r="G174" s="17" t="inlineStr">
         <is>
-          <t>Basic deployment configuration via env + launch scripts.</t>
+          <t>Deployment configuration (plan→edition).</t>
         </is>
       </c>
       <c r="H174" s="17" t="inlineStr"/>
@@ -7316,24 +7408,24 @@
           <t>14. Deployment &amp; Integration</t>
         </is>
       </c>
-      <c r="D175" s="19" t="inlineStr">
-        <is>
-          <t>Partial</t>
-        </is>
-      </c>
-      <c r="E175" s="20" t="inlineStr">
-        <is>
-          <t>~</t>
+      <c r="D175" s="23" t="inlineStr">
+        <is>
+          <t>Included</t>
+        </is>
+      </c>
+      <c r="E175" s="24" t="inlineStr">
+        <is>
+          <t>✓</t>
         </is>
       </c>
       <c r="F175" s="17" t="inlineStr">
         <is>
-          <t>env vars, qb_api</t>
+          <t>qb_saas (editions)</t>
         </is>
       </c>
       <c r="G175" s="17" t="inlineStr">
         <is>
-          <t>Minimal environment handling; no formal profiles.</t>
+          <t>Environment profiles (edition tiers).</t>
         </is>
       </c>
       <c r="H175" s="17" t="inlineStr"/>
@@ -9390,14 +9482,14 @@
         </is>
       </c>
       <c r="B13" s="26" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="C13" s="26" t="n">
         <v>1</v>
       </c>
       <c r="D13" s="27" t="inlineStr">
         <is>
-          <t>119, 120, 121, 122, 123, 124, 125, 126, 127, 129, 130</t>
+          <t>120, 127</t>
         </is>
       </c>
     </row>
@@ -9408,14 +9500,14 @@
         </is>
       </c>
       <c r="B14" s="26" t="n">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="C14" s="26" t="n">
         <v>0</v>
       </c>
       <c r="D14" s="27" t="inlineStr">
         <is>
-          <t>131, 132, 133, 134, 135, 136, 137, 138, 139, 140, 141, 142, 143, 144, 145</t>
+          <t>135, 136, 137, 138, 139, 143, 144, 145</t>
         </is>
       </c>
     </row>
@@ -9426,14 +9518,14 @@
         </is>
       </c>
       <c r="B15" s="26" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="C15" s="26" t="n">
         <v>0</v>
       </c>
       <c r="D15" s="27" t="inlineStr">
         <is>
-          <t>146, 147, 148, 149, 150, 151, 152, 153, 154, 155</t>
+          <t>148, 152, 153</t>
         </is>
       </c>
     </row>
@@ -9462,10 +9554,10 @@
         </is>
       </c>
       <c r="B17" s="26" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C17" s="26" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D17" s="27" t="inlineStr">
         <is>
@@ -9483,11 +9575,11 @@
         <v>0</v>
       </c>
       <c r="C18" s="26" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D18" s="27" t="inlineStr">
         <is>
-          <t>173, 174, 175, 176</t>
+          <t>175, 176</t>
         </is>
       </c>
     </row>

</xml_diff>